<commit_message>
Step 11: final sector note (PDF + Word)
</commit_message>
<xml_diff>
--- a/outputs/red_flag_watchlist.xlsx
+++ b/outputs/red_flag_watchlist.xlsx
@@ -5584,7 +5584,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="36.75" customHeight="1">
+    <row r="7" ht="55.125" customHeight="1">
       <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Torrent</t>
@@ -5635,7 +5635,7 @@
       </c>
       <c r="R7" s="19" t="inlineStr">
         <is>
-          <t>FY2026 debt-funded acquisition (borrowings 3,202 -&gt; 15,026 cr) drives Altman Grey, AQI and DSRI; likely acquisition artifact.</t>
+          <t>FY2026 acquisition of a 46.39% stake in JB Chemicals &amp; Pharmaceuticals (completed Jan 2026), partly bond-funded: borrowings 3,202 -&gt; 15,026 cr. Drives Altman Grey, AQI and DSRI; likely acquisition artifact.</t>
         </is>
       </c>
     </row>

</xml_diff>